<commit_message>
Vị trí các nút bấm Configurable và Power trên board
</commit_message>
<xml_diff>
--- a/Design.xlsx
+++ b/Design.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\FPGA\FPGA-DevKits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399F823B-B05F-464C-8CFE-57E6A4210F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A61376C-5E64-4E0B-818C-8497A448638F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GPIO" sheetId="1" r:id="rId1"/>
-    <sheet name="bits - hwh" sheetId="2" r:id="rId2"/>
+    <sheet name="Board" sheetId="3" r:id="rId2"/>
+    <sheet name="bits - hwh" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -738,7 +739,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -852,8 +853,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1897,6 +1896,2214 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>9208</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>172382</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>107819</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>172382</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1204F63F-9ACA-4B05-87AC-5F5AD20FCE6C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="1675" t="4935" r="2399" b="5018"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1522698" y="7713554"/>
+          <a:ext cx="7476873" cy="4782207"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>17931</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>48</xdr:col>
+      <xdr:colOff>116542</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB83221C-4FF4-F29E-09D7-91385AA138B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="1675" t="4935" r="2399" b="5018"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1712260" y="1048871"/>
+          <a:ext cx="7440706" cy="4661648"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Speech Bubble: Rectangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14BCB26D-CA05-AD1B-2ED2-E9E347770BC2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3421380" y="6111240"/>
+          <a:ext cx="1524000" cy="815340"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 31353"/>
+            <a:gd name="adj2" fmla="val -143137"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>PROG</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>Xóa cấu hình hiện tại của vùng FPGA và buộc nó phải nạp lại từ đầu.</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>180133</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>62948</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>46383</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>146767</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Speech Bubble: Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B04A5621-FE46-45B6-BE05-04683CAC86BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5176203" y="6185452"/>
+          <a:ext cx="827032" cy="825941"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -39768"/>
+            <a:gd name="adj2" fmla="val -123081"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>SRST</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>Khởi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" baseline="0"/>
+            <a:t> động lại toàn bộ Dev Kit</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>15571</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>41744</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>130188</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>112644</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Speech Bubble: Rectangle 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F5CC4FF0-1353-49C3-8F66-4CB35B7BFE1C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4050858" y="5793187"/>
+          <a:ext cx="498930" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -6864"/>
+            <a:gd name="adj2" fmla="val -112696"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>SW</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>M20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>41744</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>183197</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>112644</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Speech Bubble: Rectangle 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A61424FA-B2C3-4EC1-99F6-1A3E2320E490}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3527397" y="5793187"/>
+          <a:ext cx="498930" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>SW1</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>M19</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>15570</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>13252</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>72886</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>92766</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Speech Bubble: Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0AE33DE1-9577-4B35-AC33-10B69853CE10}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4050857" y="3909391"/>
+          <a:ext cx="1018099" cy="450575"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -36967"/>
+            <a:gd name="adj2" fmla="val 126269"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>R</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>G</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>B</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>N15</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>G17</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>L15</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>86139</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>8614</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>132523</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>86139</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Speech Bubble: Rectangle 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADDFF4F0-6723-46D7-8F58-3F815EEA987D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2968487" y="3904753"/>
+          <a:ext cx="1007166" cy="448586"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 36975"/>
+            <a:gd name="adj2" fmla="val 127791"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>R</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>G</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>B</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>1</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>M</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>15</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>L14</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>G15</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>33131</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>35117</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>185529</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>106017</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Speech Bubble: Rectangle 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DBCCD45-F25C-49F5-9CD1-30E2FCEE5B87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6566453" y="5972091"/>
+          <a:ext cx="536711" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 5356"/>
+            <a:gd name="adj2" fmla="val -118785"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN3</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>L</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>19</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>22088</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>35117</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>174486</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>106017</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Speech Bubble: Rectangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{614B1AED-9020-E5A7-9EBA-3C9455CF65CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7131879" y="5972091"/>
+          <a:ext cx="536711" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN2</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>L20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>11044</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>35117</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>163442</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>106017</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Speech Bubble: Rectangle 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{097682B0-F845-0674-55CB-2C656831B2F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7697305" y="5972091"/>
+          <a:ext cx="536711" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN1</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>35117</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>152399</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>106017</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Speech Bubble: Rectangle 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DAF187D-6E8D-EB7F-12A9-ABA06DC4CEC8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8262731" y="5972091"/>
+          <a:ext cx="536711" cy="441961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D19</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>79513</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>106018</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>183197</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Speech Bubble: Rectangle 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30D191DB-D125-4BFA-9AC8-91102806EF17}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="848139" y="4744279"/>
+          <a:ext cx="872310" cy="450574"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 127427"/>
+            <a:gd name="adj2" fmla="val 13126"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>DC1 Power</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>7v ~ 15v</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>53009</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>71438</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Speech Bubble: Rectangle 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09661C24-64FF-434F-A6C4-5D464542D95F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="815009" y="5791200"/>
+          <a:ext cx="1732929" cy="866775"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 105396"/>
+            <a:gd name="adj2" fmla="val -125238"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>JP9:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> chọn nguồn</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3  (3-2)</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Nguồn từ USB</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>2</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>1 (1-2) ==&gt;</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>  từ VIN, DC1</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>168344</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>56725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>48127</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>168442</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="Speech Bubble: Rectangle 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD5A8846-2EBB-4B91-9A69-2C72831FF1C7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6713523" y="4115378"/>
+          <a:ext cx="842309" cy="296201"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 4492"/>
+            <a:gd name="adj2" fmla="val 149032"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Nguồn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> VIN</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68180</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>120141</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>181803</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>14125</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="Speech Bubble: Rectangle 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16D6D82D-10DD-43C8-9F27-FC82F96413C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838201" y="4178794"/>
+          <a:ext cx="883644" cy="447436"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 127427"/>
+            <a:gd name="adj2" fmla="val 13126"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Micro</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> USB</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>182728</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>103239</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>54</xdr:col>
+      <xdr:colOff>102920</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>178931</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="Speech Bubble: Rectangle 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A99C74B3-7E05-407F-B875-7500664763B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9598398" y="2515135"/>
+          <a:ext cx="880974" cy="446753"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -98213"/>
+            <a:gd name="adj2" fmla="val 11643"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>JP1: Boot</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> Mode</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>22669</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>38810</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>106491</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>150982</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Speech Bubble: Rectangle 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D21E0FA1-E352-4F88-985F-1C8232411433}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4725298" y="10031896"/>
+          <a:ext cx="867593" cy="297229"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 12780"/>
+            <a:gd name="adj2" fmla="val 159602"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent3"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>CLK 50MHz</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>139709</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>61029</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>26277</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>120869</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="Speech Bubble: Rectangle 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{039DFF80-1A40-4AC5-BC83-12197554ADF9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3923433" y="10729029"/>
+          <a:ext cx="1021685" cy="611633"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 52550"/>
+            <a:gd name="adj2" fmla="val 83322"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent3"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>IC nguồn 4 kênh</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> độc lập TPS65400</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>181751</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>61029</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>68319</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>21021</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Speech Bubble: Rectangle 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0ED68FA-22B6-44D1-90FB-7DBE8050679B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3019544" y="9993305"/>
+          <a:ext cx="1021685" cy="511785"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -36435"/>
+            <a:gd name="adj2" fmla="val 85040"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent3"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>Giao tiếp</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" b="1" baseline="0"/>
+            <a:t> USB</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>FT2232HQ</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>59457</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>138657</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>120870</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>47295</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="Speech Bubble: Rectangle 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF68CF06-6FFE-DB55-1FF5-19EB80914DD8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5545857" y="9151278"/>
+          <a:ext cx="1007344" cy="460431"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 12780"/>
+            <a:gd name="adj2" fmla="val 71717"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent3"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>RAM</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>DDL 512MB</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>60881</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>176641</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>136635</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>136633</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="Speech Bubble: Rectangle 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6842D58C-80B7-4642-9CFC-BD927611C8DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3277047" y="8821400"/>
+          <a:ext cx="1021685" cy="511785"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -72440"/>
+            <a:gd name="adj2" fmla="val -23804"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent3"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent3"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>Audio Codec</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>ADAU</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" b="1" baseline="0"/>
+            <a:t> 1761</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>2056</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>146003</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>105741</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>39986</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="Speech Bubble: Rectangle 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B85A35BF-42DE-4076-A55B-8982972B877F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1515546" y="5296072"/>
+          <a:ext cx="860429" cy="445776"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 179953"/>
+            <a:gd name="adj2" fmla="val -166064"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Led</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> đỏ </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>báo nguồn</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -3561,6 +5768,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968AC48A-2378-4E91-8413-C6C5E438A215}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="2.77734375" defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C38D68DB-870D-4233-B871-A8BC2088FA29}">
   <dimension ref="B2:AL19"/>
   <sheetFormatPr defaultColWidth="2.77734375" defaultRowHeight="14.4"/>
@@ -3606,10 +5823,10 @@
     </row>
     <row r="3" spans="2:38">
       <c r="B3" s="68"/>
-      <c r="C3" s="98" t="s">
+      <c r="C3" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="99"/>
+      <c r="D3" s="70"/>
       <c r="E3" s="71"/>
       <c r="J3" s="46"/>
       <c r="X3" s="65" t="s">
@@ -3761,11 +5978,11 @@
     <row r="11" spans="2:38">
       <c r="B11" s="89"/>
       <c r="C11" s="90"/>
-      <c r="D11" s="100" t="s">
+      <c r="D11" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="101"/>
-      <c r="F11" s="102"/>
+      <c r="E11" s="99"/>
+      <c r="F11" s="100"/>
       <c r="J11" s="46"/>
       <c r="X11" s="83"/>
       <c r="Y11" s="84" t="s">

</xml_diff>